<commit_message>
Yumuşatma ikinci turu ve netlik: yazı tipleri, okur dili düzeltmeleri
Özel depodaki ab7d368'in yayın kopyası. Hinting'li yazı tipleri ve çubukta canlı
logo yazısı; iz taramasındaki 27 bulgunun düzeltmesi (başlıklar, notlar, reform
modelleri hücreleri, mutabakat notları); veri sürümü 20 Ekim 2026 (sayılar aynı:
266 öneri, 322 ret oyu); site haritası lastmod 20 Ekim. README girişi güncellendi,
.gitignore'a yazı tipi kaynakları eklendi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/web/veri/vetolar.xlsx
+++ b/web/veri/vetolar.xlsx
@@ -1141,12 +1141,12 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (scprocedure #8).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (Tablo 4, #8).</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (scprocedure #8).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (Table 4, #8).</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1232,12 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (scprocedure #7).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (Tablo 4, #7).</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (scprocedure #7).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (Table 4, #7).</t>
         </is>
       </c>
     </row>
@@ -1323,12 +1323,12 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (scprocedure #6).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (Tablo 4, #6).</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (scprocedure #6).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (Table 4, #6).</t>
         </is>
       </c>
     </row>
@@ -1687,12 +1687,12 @@
       </c>
       <c r="Z13" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (scprocedure #14).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (Tablo 4, #14).</t>
         </is>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (scprocedure #14).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (Table 4, #14).</t>
         </is>
       </c>
     </row>
@@ -1778,12 +1778,12 @@
       </c>
       <c r="Z14" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (scprocedure #13).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (Tablo 4, #13).</t>
         </is>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (scprocedure #13).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (Table 4, #13).</t>
         </is>
       </c>
     </row>
@@ -1869,12 +1869,12 @@
       </c>
       <c r="Z15" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (scprocedure #12).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün üç üyelik vetosu; ülke adına göre eşleştirildi (Tablo 4, #12).</t>
         </is>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (scprocedure #12).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Three membership vetoes on the same day; matched by country name (Table 4, #12).</t>
         </is>
       </c>
     </row>
@@ -2152,12 +2152,12 @@
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün iki üyelik vetosu; ülke adına göre eşleştirildi (scprocedure #18).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün iki üyelik vetosu; ülke adına göre eşleştirildi (Tablo 4, #18).</t>
         </is>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Two membership vetoes on the same day; matched by country name (scprocedure #18).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Two membership vetoes on the same day; matched by country name (Table 4, #18).</t>
         </is>
       </c>
     </row>
@@ -2243,12 +2243,12 @@
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün iki üyelik vetosu; ülke adına göre eşleştirildi (scprocedure #17).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Aynı gün iki üyelik vetosu; ülke adına göre eşleştirildi (Tablo 4, #17).</t>
         </is>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Two membership vetoes on the same day; matched by country name (scprocedure #17).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: Two membership vetoes on the same day; matched by country name (Table 4, #17).</t>
         </is>
       </c>
     </row>
@@ -2890,12 +2890,12 @@
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: scprocedure dipnot 9: esas taslağa yönelik ikinci veto (#26) (scprocedure #26).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Oy dağılımı: Referans tablonun 9. dipnotuna göre esas taslağa yönelik ikinci veto (Tablo 4, #26).</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: scprocedure footnote 9: second veto, on the substantive draft (#26) (scprocedure #26).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Vote breakdown: According to footnote 9 of the reference table, the second veto, on the substantive draft (Table 4, #26).</t>
         </is>
       </c>
     </row>
@@ -2981,12 +2981,12 @@
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Ön soru vetosu: konunun usul meselesi sayılıp sayılmayacağına dair oylama (çifte veto). | Oy dağılımı: scprocedure dipnot 9: bu toplantıdaki ilk veto ön soru vetosudur (#25) (scprocedure #25).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Taslak ayrı belge olarak yayımlanmamış; öneri toplantı kaydında yer alıyor. | Ön soru vetosu: konunun usul meselesi sayılıp sayılmayacağına dair oylama (çifte veto). | Oy dağılımı: Referans tablonun 9. dipnotuna göre bu toplantıdaki ilk veto ön soru vetosudur (Tablo 4, #25).</t>
         </is>
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Preliminary-question veto: vote on whether the matter is to be considered procedural (double veto). | Vote breakdown: scprocedure footnote 9: the first veto at this meeting is a preliminary-question veto (#25) (scprocedure #25).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | The draft was not issued as a separate document; the proposal appears in the meeting record. | Preliminary-question veto: vote on whether the matter is to be considered procedural (double veto). | Vote breakdown: According to footnote 9 of the reference table, the first veto at this meeting is a preliminary-question veto (Table 4, #25).</t>
         </is>
       </c>
     </row>
@@ -4648,12 +4648,12 @@
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Oy dağılımı 9-2-0: S/PV.456 PDF s. 36: Kanada taslağı S/1431 Arjantin'in isteğiyle iki parça hâlinde oylandı; son paragraf dışındaki bölüm 9 lehte, 2 aleyhte (Ukrayna SSC, SSCB). Referans tablo bu vetoya da 8-2-1 veriyor; toplantı kaydında Arjantin bu oylamada lehte. DHL'deki iki satır birbirinin aynısı; kimlikler toplantıdaki oylama sırasına göre bağlandı. | scprocedure Tablo 4 #43 oy dağılımını 8-2-1 veriyor; toplantı kaydı esas alındı.</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Oy dağılımı 9-2-0: S/PV.456 PDF s. 36: Kanada taslağı S/1431 Arjantin'in isteğiyle iki parça hâlinde oylandı; son paragraf dışındaki bölüm 9 lehte, 2 aleyhte (Ukrayna SSC, SSCB). Referans tablo bu vetoya da 8-2-1 veriyor; toplantı kaydında Arjantin bu oylamada lehte. DHL'deki iki satır birbirinin aynısı; kimlikler toplantıdaki oylama sırasına göre bağlandı. | Referans tablo (Tablo 4, #43) oy dağılımını 8-2-1 veriyor; toplantı kaydı esas alındı.</t>
         </is>
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | Vote breakdown 9-2-0: S/PV.456 PDF p. 36: the Canadian draft S/1431 was voted on in two parts at the request of Argentina; the part other than the last paragraph 9 in favour, 2 against (Ukrainian SSR, USSR). The reference table also gives 8-2-1 for this veto; in the meeting record Argentina voted in favour in this vote. The two lines in the DHL list are identical; the identifiers were assigned in the order of the votes at the meeting. | scprocedure Table 4 #43 gives the vote breakdown as 8-2-1; the meeting record was followed.</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | Vote breakdown 9-2-0: S/PV.456 PDF p. 36: the Canadian draft S/1431 was voted on in two parts at the request of Argentina; the part other than the last paragraph 9 in favour, 2 against (Ukrainian SSR, USSR). The reference table also gives 8-2-1 for this veto; in the meeting record Argentina voted in favour in this vote. The two lines in the DHL list are identical; the identifiers were assigned in the order of the votes at the meeting. | The reference table (Table 4, #43) gives the vote breakdown as 8-2-1; the meeting record was followed.</t>
         </is>
       </c>
     </row>
@@ -9315,12 +9315,12 @@
       </c>
       <c r="Z90" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Oy dağılımı: Aynı gün iki üyelik vetosu; ülke adına göre eşleştirildi (scprocedure #90).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Oy dağılımı: Aynı gün iki üyelik vetosu; ülke adına göre eşleştirildi (Tablo 4, #90).</t>
         </is>
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | Vote breakdown: Two membership vetoes on the same day; matched by country name (scprocedure #90).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | Vote breakdown: Two membership vetoes on the same day; matched by country name (Table 4, #90).</t>
         </is>
       </c>
     </row>
@@ -9411,12 +9411,12 @@
       </c>
       <c r="Z91" t="inlineStr">
         <is>
-          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Oy dağılımı: Aynı gün iki üyelik vetosu; ülke adına göre eşleştirildi (scprocedure #89).</t>
+          <t>SSCB vetosu; Rusya Federasyonu koltuğun halefidir, analizde ayrı tutulur. | Oy dağılımı: Aynı gün iki üyelik vetosu; ülke adına göre eşleştirildi (Tablo 4, #89).</t>
         </is>
       </c>
       <c r="AA91" t="inlineStr">
         <is>
-          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | Vote breakdown: Two membership vetoes on the same day; matched by country name (scprocedure #89).</t>
+          <t>USSR veto; the Russian Federation is the successor to the seat and is kept separate in the analysis. | Vote breakdown: Two membership vetoes on the same day; matched by country name (Table 4, #89).</t>
         </is>
       </c>
     </row>
@@ -15334,12 +15334,12 @@
       </c>
       <c r="Z154" t="inlineStr">
         <is>
-          <t>Oy dağılımı: Aynı gün iki farklı gündem; konuya göre eşleştirildi (scprocedure #154).</t>
+          <t>Oy dağılımı: Aynı gün iki farklı gündem; konuya göre eşleştirildi (Tablo 4, #154).</t>
         </is>
       </c>
       <c r="AA154" t="inlineStr">
         <is>
-          <t>Vote breakdown: Two different agenda items on the same day; matched by subject (scprocedure #154).</t>
+          <t>Vote breakdown: Two different agenda items on the same day; matched by subject (Table 4, #154).</t>
         </is>
       </c>
     </row>
@@ -15430,12 +15430,12 @@
       </c>
       <c r="Z155" t="inlineStr">
         <is>
-          <t>Oy dağılımı: Aynı gün iki farklı gündem; konuya göre eşleştirildi (scprocedure #153).</t>
+          <t>Oy dağılımı: Aynı gün iki farklı gündem; konuya göre eşleştirildi (Tablo 4, #153).</t>
         </is>
       </c>
       <c r="AA155" t="inlineStr">
         <is>
-          <t>Vote breakdown: Two different agenda items on the same day; matched by subject (scprocedure #153).</t>
+          <t>Vote breakdown: Two different agenda items on the same day; matched by subject (Table 4, #153).</t>
         </is>
       </c>
     </row>
@@ -21621,12 +21621,12 @@
       </c>
       <c r="Z225" t="inlineStr">
         <is>
-          <t>Oy dağılımı 10-1-4: S/PV.7481 PDF s. 7: S/2015/508; 10 lehte, 1 aleyhte (Rusya), 4 çekimser (Angola, Çin, Nijerya, Venezuela). | scprocedure Tablo 4 #224 oy dağılımını 11-1-4 veriyor; toplantı kaydı esas alındı.</t>
+          <t>Oy dağılımı 10-1-4: S/PV.7481 PDF s. 7: S/2015/508; 10 lehte, 1 aleyhte (Rusya), 4 çekimser (Angola, Çin, Nijerya, Venezuela). | Referans tablo (Tablo 4, #224) oy dağılımını 11-1-4 veriyor; toplantı kaydı esas alındı.</t>
         </is>
       </c>
       <c r="AA225" t="inlineStr">
         <is>
-          <t>Vote breakdown 10-1-4: S/PV.7481 PDF p. 7: S/2015/508; 10 in favour, 1 against (Russia), 4 abstaining (Angola, China, Nigeria, Venezuela). | scprocedure Table 4 #224 gives the vote breakdown as 11-1-4; the meeting record was followed.</t>
+          <t>Vote breakdown 10-1-4: S/PV.7481 PDF p. 7: S/2015/508; 10 in favour, 1 against (Russia), 4 abstaining (Angola, China, Nigeria, Venezuela). | The reference table (Table 4, #224) gives the vote breakdown as 11-1-4; the meeting record was followed.</t>
         </is>
       </c>
     </row>
@@ -23265,12 +23265,12 @@
       </c>
       <c r="Z244" t="inlineStr">
         <is>
-          <t>Oy dağılımı 12-2-1: S/PV.8926 PDF s. 5: S/2021/990; 12 lehte, 2 aleyhte (Hindistan, Rusya), 1 çekimser (Çin). | scprocedure Tablo 4 #243 oy dağılımını 13-2-1 veriyor; toplantı kaydı esas alındı.</t>
+          <t>Oy dağılımı 12-2-1: S/PV.8926 PDF s. 5: S/2021/990; 12 lehte, 2 aleyhte (Hindistan, Rusya), 1 çekimser (Çin). | Referans tablo (Tablo 4, #243) oy dağılımını 13-2-1 veriyor; toplantı kaydı esas alındı.</t>
         </is>
       </c>
       <c r="AA244" t="inlineStr">
         <is>
-          <t>Vote breakdown 12-2-1: S/PV.8926 PDF p. 5: S/2021/990; 12 in favour, 2 against (India, Russia), 1 abstaining (China). | scprocedure Table 4 #243 gives the vote breakdown as 13-2-1; the meeting record was followed.</t>
+          <t>Vote breakdown 12-2-1: S/PV.8926 PDF p. 5: S/2021/990; 12 in favour, 2 against (India, Russia), 1 abstaining (China). | The reference table (Table 4, #243) gives the vote breakdown as 13-2-1; the meeting record was followed.</t>
         </is>
       </c>
     </row>
@@ -25457,12 +25457,12 @@
       </c>
       <c r="Z266" t="inlineStr">
         <is>
-          <t>Oy dağılımı 11-2-2: DHL'de oy dağılımı yok, referans tablo Eylül 2025'te bitiyor. S/PV.10130 s. 4: S/2026/273 (Bahreyn, Ürdün, Kuveyt, Katar, Suudi Arabistan ve BAE taslağı, Hürmüz Boğazı) 11 lehte, 2 aleyhte (Çin, Rusya Federasyonu), 2 çekimser (Kolombiya, Pakistan). Kayıtta Başkan 'bir daimi üyenin ret oyu nedeniyle' diyor; oy listesinde iki daimi üye aleyhte. Basın bülteni SC/16330 (https://press.un.org/en/2026/sc16330.doc.htm) press.un.org CAPTCHA istediği için açılamadı; numara doğrulanamadı.</t>
+          <t>Oy dağılımı 11-2-2: DHL listesinde oy dağılımı yok, referans tablo bu tarihi kapsamıyor. S/PV.10130 s. 4: S/2026/273 (Bahreyn, Ürdün, Kuveyt, Katar, Suudi Arabistan ve BAE taslağı, Hürmüz Boğazı) 11 lehte, 2 aleyhte (Çin, Rusya Federasyonu), 2 çekimser (Kolombiya, Pakistan). Kayıtta Başkan 'bir daimi üyenin ret oyu nedeniyle' diyor; oy listesinde iki daimi üye aleyhte. Basın bülteni SC/16330 (https://press.un.org/en/2026/sc16330.doc.htm) doğrulanamadı.</t>
         </is>
       </c>
       <c r="AA266" t="inlineStr">
         <is>
-          <t>Vote breakdown 11-2-2: The DHL list has no vote breakdown; the reference table ends in September 2025. S/PV.10130 p. 4: S/2026/273 (draft by Bahrain, Jordan, Kuwait, Qatar, Saudi Arabia and the UAE, Strait of Hormuz) 11 in favour, 2 against (China, Russian Federation), 2 abstaining (Colombia, Pakistan). In the record the President refers to the negative vote of a permanent member; in the voting list two permanent members voted against. Press release SC/16330 (https://press.un.org/en/2026/sc16330.doc.htm) could not be opened because press.un.org required a CAPTCHA; the number could not be verified.</t>
+          <t>Vote breakdown 11-2-2: The DHL list has no vote breakdown and the reference table does not cover this date. S/PV.10130 p. 4: S/2026/273 (draft by Bahrain, Jordan, Kuwait, Qatar, Saudi Arabia and the UAE, Strait of Hormuz) 11 in favour, 2 against (China, Russian Federation), 2 abstaining (Colombia, Pakistan). In the record the President refers to the negative vote of a permanent member; in the voting list two permanent members voted against. Press release SC/16330 (https://press.un.org/en/2026/sc16330.doc.htm) could not be verified.</t>
         </is>
       </c>
     </row>
@@ -25578,12 +25578,12 @@
       </c>
       <c r="Z267" t="inlineStr">
         <is>
-          <t>DHL listesinde yok (10 Ekim 2026 indirmesi), referans tablo Eylül 2025'te bitiyor. S/PV.10224 s. 4: S/2026/740 (ABD taslağı) 11 lehte, 2 aleyhte (Çin, Rusya Federasyonu), 2 çekimser (Pakistan, Somali); kabul edilmedi. Taslak, 1929 (2010) sayılı kararın 29. paragrafıyla kurulan ve İran yaptırımlarını izleyen Uzmanlar Paneli'nin görevini uzatıyordu. Toplantı başında gündemin kabulü 11-2-2 usul oylamasıyla geçti (usul oylamasında veto yoktur). Basın bülteni SC/16455 (https://press.un.org/en/2026/sc16455.doc.htm) aynı sonucu veriyor.</t>
+          <t>DHL listesinde ve referans tabloda henüz yok. S/PV.10224 s. 4: S/2026/740 (ABD taslağı) 11 lehte, 2 aleyhte (Çin, Rusya Federasyonu), 2 çekimser (Pakistan, Somali); kabul edilmedi. Taslak, 1929 (2010) sayılı kararın 29. paragrafıyla kurulan ve İran yaptırımlarını izleyen Uzmanlar Paneli'nin görevini uzatıyordu. Toplantı başında gündemin kabulü 11-2-2 usul oylamasıyla geçti (usul oylamasında veto yoktur). Basın bülteni SC/16455 (https://press.un.org/en/2026/sc16455.doc.htm) aynı sonucu veriyor.</t>
         </is>
       </c>
       <c r="AA267" t="inlineStr">
         <is>
-          <t>Not in the DHL list (download of 10 October 2026); the reference table ends in September 2025. S/PV.10224 p. 4: S/2026/740 (United States draft) 11 in favour, 2 against (China, Russian Federation), 2 abstaining (Pakistan, Somalia); not adopted. The draft would have extended the mandate of the Panel of Experts established by paragraph 29 of resolution 1929 (2010) to monitor the sanctions on Iran. At the start of the meeting the agenda was adopted by a procedural vote of 11-2-2 (there is no veto in procedural votes). Press release SC/16455 (https://press.un.org/en/2026/sc16455.doc.htm) gives the same result.</t>
+          <t>Not yet in the DHL list or the reference table. S/PV.10224 p. 4: S/2026/740 (United States draft) 11 in favour, 2 against (China, Russian Federation), 2 abstaining (Pakistan, Somalia); not adopted. The draft would have extended the mandate of the Panel of Experts established by paragraph 29 of resolution 1929 (2010) to monitor the sanctions on Iran. At the start of the meeting the agenda was adopted by a procedural vote of 11-2-2 (there is no veto in procedural votes). Press release SC/16455 (https://press.un.org/en/2026/sc16455.doc.htm) gives the same result.</t>
         </is>
       </c>
     </row>

</xml_diff>